<commit_message>
fix: rebuild all sheets with inline dropdowns and corrected CF formulas
- attendance_monthly: 4-row header, H\$3 CF pattern for weekend/empty detection, SUMPRODUCT consecutive absence rule, inline dropdown
- employees_database: removed hidden 'قوائم' sheet, all dropdowns now inline lists
- attendance_tracker: fixed MergedCell error, clean row structure with status dropdown and CF

https://claude.ai/code/session_016xio8QrybJF7hs3vMN83gG
</commit_message>
<xml_diff>
--- a/attendance_tracker.xlsx
+++ b/attendance_tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="سجل الحضور" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'سجل الحضور'!$2:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'سجل الحضور'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="HH:MM"/>
     <numFmt numFmtId="166" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,7 +35,7 @@
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="24"/>
+      <sz val="22"/>
     </font>
     <font>
       <name val="Cairo"/>
@@ -45,11 +45,6 @@
     </font>
     <font>
       <name val="Cairo"/>
-      <color rgb="001F3864"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Cairo"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="13"/>
@@ -64,12 +59,11 @@
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Cairo"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001F3864"/>
       <sz val="12"/>
     </font>
     <font>
@@ -79,19 +73,19 @@
     </font>
     <font>
       <name val="Cairo"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Cairo"/>
       <color rgb="00555555"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Cairo"/>
@@ -108,47 +102,41 @@
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="001565C0"/>
-      <sz val="16"/>
+      <color rgb="001B5E20"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="002E7D32"/>
-      <sz val="16"/>
+      <color rgb="00B71C1C"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="00C62828"/>
-      <sz val="16"/>
+      <color rgb="001565C0"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="00BF360C"/>
-      <sz val="16"/>
+      <color rgb="00555555"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
-      <color rgb="004A148C"/>
-      <sz val="16"/>
+      <color rgb="00804000"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00827717"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Cairo"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="10"/>
+      <sz val="15"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -167,17 +155,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DEEAF1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFDE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
@@ -187,7 +175,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BBDEFB"/>
+        <fgColor rgb="00EEF4FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -207,21 +195,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDE7F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -231,16 +214,16 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="002E75B6"/>
+        <color rgb="00FFFFFF"/>
       </left>
       <right style="medium">
-        <color rgb="002E75B6"/>
+        <color rgb="00FFFFFF"/>
       </right>
       <top style="medium">
-        <color rgb="002E75B6"/>
+        <color rgb="00FFFFFF"/>
       </top>
       <bottom style="medium">
-        <color rgb="002E75B6"/>
+        <color rgb="00FFFFFF"/>
       </bottom>
     </border>
     <border>
@@ -272,6 +255,48 @@
       </bottom>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="001F3864"/>
+      </left>
+      <right style="medium">
+        <color rgb="001F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F3864"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002E75B6"/>
+      </left>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="003A5F8F"/>
+      </left>
+      <right style="thin">
+        <color rgb="003A5F8F"/>
+      </right>
+      <top style="thin">
+        <color rgb="003A5F8F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="003A5F8F"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="00CCCCCC"/>
       </left>
@@ -286,17 +311,31 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00AAAAAA"/>
+      <left style="medium">
+        <color rgb="001B5E20"/>
       </left>
-      <right style="thin">
-        <color rgb="00AAAAAA"/>
+      <right style="medium">
+        <color rgb="001B5E20"/>
       </right>
-      <top style="thin">
-        <color rgb="00AAAAAA"/>
+      <top style="medium">
+        <color rgb="001B5E20"/>
       </top>
-      <bottom style="thin">
-        <color rgb="00AAAAAA"/>
+      <bottom style="medium">
+        <color rgb="001B5E20"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00B71C1C"/>
+      </left>
+      <right style="medium">
+        <color rgb="00B71C1C"/>
+      </right>
+      <top style="medium">
+        <color rgb="00B71C1C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00B71C1C"/>
       </bottom>
     </border>
     <border>
@@ -315,58 +354,30 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="002E7D32"/>
+        <color rgb="00555555"/>
       </left>
       <right style="medium">
-        <color rgb="002E7D32"/>
+        <color rgb="00555555"/>
       </right>
       <top style="medium">
-        <color rgb="002E7D32"/>
+        <color rgb="00555555"/>
       </top>
       <bottom style="medium">
-        <color rgb="002E7D32"/>
+        <color rgb="00555555"/>
       </bottom>
     </border>
     <border>
       <left style="medium">
-        <color rgb="00C62828"/>
+        <color rgb="00804000"/>
       </left>
       <right style="medium">
-        <color rgb="00C62828"/>
+        <color rgb="00804000"/>
       </right>
       <top style="medium">
-        <color rgb="00C62828"/>
+        <color rgb="00804000"/>
       </top>
       <bottom style="medium">
-        <color rgb="00C62828"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00BF360C"/>
-      </left>
-      <right style="medium">
-        <color rgb="00BF360C"/>
-      </right>
-      <top style="medium">
-        <color rgb="00BF360C"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00BF360C"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="004A148C"/>
-      </left>
-      <right style="medium">
-        <color rgb="004A148C"/>
-      </right>
-      <top style="medium">
-        <color rgb="004A148C"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="004A148C"/>
+        <color rgb="00804000"/>
       </bottom>
     </border>
     <border>
@@ -383,20 +394,6 @@
         <color rgb="00827717"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00DDDDDD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00DDDDDD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00DDDDDD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00DDDDDD"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -409,92 +406,92 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="14" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="18" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -506,6 +503,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFE0E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EEEEEE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -533,14 +537,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E8E8E8"/>
+          <fgColor rgb="00ECECEC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <fgColor rgb="00F8F8F8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -903,132 +907,183 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E75B6"/>
+    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H49"/>
+  <dimension ref="B1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="3" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
-    <row r="2" ht="54" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="1" ht="54" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>سجل حضور وانصراف الموظفين</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="34" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>الشهر</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4">
+        <f>CHOOSE(C2,"يناير","فبراير","مارس","أبريل","مايو","يونيو","يوليو","أغسطس","سبتمبر","أكتوبر","نوفمبر","ديسمبر")</f>
+        <v/>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>السنة</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G2" s="5">
+        <f>D2&amp;"  "&amp; F2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>اسم الموظف</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>القسم / الوظيفة</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>الشهر</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5">
-        <f>CHOOSE(C5,"يناير","فبراير","مارس","أبريل","مايو","يونيو","يوليو","أغسطس","سبتمبر","أكتوبر","نوفمبر","ديسمبر")</f>
-        <v/>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>السنة</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G5" s="6">
-        <f>D5&amp;"  |  "&amp;F5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="8" customHeight="1"/>
-    <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="C3" s="6" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>الوظيفة / القسم</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>اليوم</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>وقت الدخول</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>وقت الخروج</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>ساعات العمل</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>الحالة</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>ملاحظات</t>
         </is>
       </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="8">
+        <f>DATE($F$2,$C$2,1)</f>
+        <v/>
+      </c>
+      <c r="C5" s="9">
+        <f>IF(B5="","",CHOOSE(WEEKDAY(B5,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="11">
+        <f>IF(AND(D5&lt;&gt;"",E5&lt;&gt;""),E5-D5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="12" t="n"/>
+      <c r="H5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="8">
+        <f>IF(B5="","",IF(MONTH(B5+1)=$C$2,B5+1,""))</f>
+        <v/>
+      </c>
+      <c r="C6" s="9">
+        <f>IF(B6="","",CHOOSE(WEEKDAY(B6,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
+        <v/>
+      </c>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="11">
+        <f>IF(AND(D6&lt;&gt;"",E6&lt;&gt;""),E6-D6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="16" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="8">
+        <f>IF(B6="","",IF(MONTH(B6+1)=$C$2,B6+1,""))</f>
+        <v/>
+      </c>
+      <c r="C7" s="9">
+        <f>IF(B7="","",CHOOSE(WEEKDAY(B7,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
+        <v/>
+      </c>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="11">
+        <f>IF(AND(D7&lt;&gt;"",E7&lt;&gt;""),E7-D7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="13" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="8">
-        <f>DATE($F$5,$C$5,1)</f>
+        <f>IF(B7="","",IF(MONTH(B7+1)=$C$2,B7+1,""))</f>
         <v/>
       </c>
       <c r="C8" s="9">
         <f>IF(B8="","",CHOOSE(WEEKDAY(B8,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
       <c r="F8" s="11">
         <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),E8-D8,"")</f>
         <v/>
       </c>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="13" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="16" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="8">
-        <f>IF(B8="","",IF(MONTH(B8+1)=$C$5,B8+1,""))</f>
+        <f>IF(B8="","",IF(MONTH(B8+1)=$C$2,B8+1,""))</f>
         <v/>
       </c>
       <c r="C9" s="9">
@@ -1046,25 +1101,25 @@
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="8">
-        <f>IF(B9="","",IF(MONTH(B9+1)=$C$5,B9+1,""))</f>
+        <f>IF(B9="","",IF(MONTH(B9+1)=$C$2,B9+1,""))</f>
         <v/>
       </c>
       <c r="C10" s="9">
         <f>IF(B10="","",CHOOSE(WEEKDAY(B10,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
       <c r="F10" s="11">
         <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),E10-D10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="13" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="16" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="8">
-        <f>IF(B10="","",IF(MONTH(B10+1)=$C$5,B10+1,""))</f>
+        <f>IF(B10="","",IF(MONTH(B10+1)=$C$2,B10+1,""))</f>
         <v/>
       </c>
       <c r="C11" s="9">
@@ -1082,25 +1137,25 @@
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="8">
-        <f>IF(B11="","",IF(MONTH(B11+1)=$C$5,B11+1,""))</f>
+        <f>IF(B11="","",IF(MONTH(B11+1)=$C$2,B11+1,""))</f>
         <v/>
       </c>
       <c r="C12" s="9">
         <f>IF(B12="","",CHOOSE(WEEKDAY(B12,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
       <c r="F12" s="11">
         <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),E12-D12,"")</f>
         <v/>
       </c>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="13" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="16" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="8">
-        <f>IF(B12="","",IF(MONTH(B12+1)=$C$5,B12+1,""))</f>
+        <f>IF(B12="","",IF(MONTH(B12+1)=$C$2,B12+1,""))</f>
         <v/>
       </c>
       <c r="C13" s="9">
@@ -1118,25 +1173,25 @@
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="8">
-        <f>IF(B13="","",IF(MONTH(B13+1)=$C$5,B13+1,""))</f>
+        <f>IF(B13="","",IF(MONTH(B13+1)=$C$2,B13+1,""))</f>
         <v/>
       </c>
       <c r="C14" s="9">
         <f>IF(B14="","",CHOOSE(WEEKDAY(B14,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
       <c r="F14" s="11">
         <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),E14-D14,"")</f>
         <v/>
       </c>
-      <c r="G14" s="12" t="n"/>
-      <c r="H14" s="13" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="16" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="8">
-        <f>IF(B14="","",IF(MONTH(B14+1)=$C$5,B14+1,""))</f>
+        <f>IF(B14="","",IF(MONTH(B14+1)=$C$2,B14+1,""))</f>
         <v/>
       </c>
       <c r="C15" s="9">
@@ -1154,25 +1209,25 @@
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="8">
-        <f>IF(B15="","",IF(MONTH(B15+1)=$C$5,B15+1,""))</f>
+        <f>IF(B15="","",IF(MONTH(B15+1)=$C$2,B15+1,""))</f>
         <v/>
       </c>
       <c r="C16" s="9">
         <f>IF(B16="","",CHOOSE(WEEKDAY(B16,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
       <c r="F16" s="11">
         <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),E16-D16,"")</f>
         <v/>
       </c>
-      <c r="G16" s="12" t="n"/>
-      <c r="H16" s="13" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="16" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="8">
-        <f>IF(B16="","",IF(MONTH(B16+1)=$C$5,B16+1,""))</f>
+        <f>IF(B16="","",IF(MONTH(B16+1)=$C$2,B16+1,""))</f>
         <v/>
       </c>
       <c r="C17" s="9">
@@ -1190,25 +1245,25 @@
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="8">
-        <f>IF(B17="","",IF(MONTH(B17+1)=$C$5,B17+1,""))</f>
+        <f>IF(B17="","",IF(MONTH(B17+1)=$C$2,B17+1,""))</f>
         <v/>
       </c>
       <c r="C18" s="9">
         <f>IF(B18="","",CHOOSE(WEEKDAY(B18,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="n"/>
       <c r="F18" s="11">
         <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),E18-D18,"")</f>
         <v/>
       </c>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="13" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="16" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="8">
-        <f>IF(B18="","",IF(MONTH(B18+1)=$C$5,B18+1,""))</f>
+        <f>IF(B18="","",IF(MONTH(B18+1)=$C$2,B18+1,""))</f>
         <v/>
       </c>
       <c r="C19" s="9">
@@ -1226,25 +1281,25 @@
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="B20" s="8">
-        <f>IF(B19="","",IF(MONTH(B19+1)=$C$5,B19+1,""))</f>
+        <f>IF(B19="","",IF(MONTH(B19+1)=$C$2,B19+1,""))</f>
         <v/>
       </c>
       <c r="C20" s="9">
         <f>IF(B20="","",CHOOSE(WEEKDAY(B20,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
       <c r="F20" s="11">
         <f>IF(AND(D20&lt;&gt;"",E20&lt;&gt;""),E20-D20,"")</f>
         <v/>
       </c>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="16" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="8">
-        <f>IF(B20="","",IF(MONTH(B20+1)=$C$5,B20+1,""))</f>
+        <f>IF(B20="","",IF(MONTH(B20+1)=$C$2,B20+1,""))</f>
         <v/>
       </c>
       <c r="C21" s="9">
@@ -1262,25 +1317,25 @@
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="B22" s="8">
-        <f>IF(B21="","",IF(MONTH(B21+1)=$C$5,B21+1,""))</f>
+        <f>IF(B21="","",IF(MONTH(B21+1)=$C$2,B21+1,""))</f>
         <v/>
       </c>
       <c r="C22" s="9">
         <f>IF(B22="","",CHOOSE(WEEKDAY(B22,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
       <c r="F22" s="11">
         <f>IF(AND(D22&lt;&gt;"",E22&lt;&gt;""),E22-D22,"")</f>
         <v/>
       </c>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="13" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="16" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="8">
-        <f>IF(B22="","",IF(MONTH(B22+1)=$C$5,B22+1,""))</f>
+        <f>IF(B22="","",IF(MONTH(B22+1)=$C$2,B22+1,""))</f>
         <v/>
       </c>
       <c r="C23" s="9">
@@ -1298,25 +1353,25 @@
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="B24" s="8">
-        <f>IF(B23="","",IF(MONTH(B23+1)=$C$5,B23+1,""))</f>
+        <f>IF(B23="","",IF(MONTH(B23+1)=$C$2,B23+1,""))</f>
         <v/>
       </c>
       <c r="C24" s="9">
         <f>IF(B24="","",CHOOSE(WEEKDAY(B24,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
       <c r="F24" s="11">
         <f>IF(AND(D24&lt;&gt;"",E24&lt;&gt;""),E24-D24,"")</f>
         <v/>
       </c>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="13" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="16" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="8">
-        <f>IF(B24="","",IF(MONTH(B24+1)=$C$5,B24+1,""))</f>
+        <f>IF(B24="","",IF(MONTH(B24+1)=$C$2,B24+1,""))</f>
         <v/>
       </c>
       <c r="C25" s="9">
@@ -1334,25 +1389,25 @@
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="8">
-        <f>IF(B25="","",IF(MONTH(B25+1)=$C$5,B25+1,""))</f>
+        <f>IF(B25="","",IF(MONTH(B25+1)=$C$2,B25+1,""))</f>
         <v/>
       </c>
       <c r="C26" s="9">
         <f>IF(B26="","",CHOOSE(WEEKDAY(B26,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
       <c r="F26" s="11">
         <f>IF(AND(D26&lt;&gt;"",E26&lt;&gt;""),E26-D26,"")</f>
         <v/>
       </c>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="13" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="16" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="8">
-        <f>IF(B26="","",IF(MONTH(B26+1)=$C$5,B26+1,""))</f>
+        <f>IF(B26="","",IF(MONTH(B26+1)=$C$2,B26+1,""))</f>
         <v/>
       </c>
       <c r="C27" s="9">
@@ -1370,25 +1425,25 @@
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="B28" s="8">
-        <f>IF(B27="","",IF(MONTH(B27+1)=$C$5,B27+1,""))</f>
+        <f>IF(B27="","",IF(MONTH(B27+1)=$C$2,B27+1,""))</f>
         <v/>
       </c>
       <c r="C28" s="9">
         <f>IF(B28="","",CHOOSE(WEEKDAY(B28,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="14" t="n"/>
       <c r="F28" s="11">
         <f>IF(AND(D28&lt;&gt;"",E28&lt;&gt;""),E28-D28,"")</f>
         <v/>
       </c>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="16" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="B29" s="8">
-        <f>IF(B28="","",IF(MONTH(B28+1)=$C$5,B28+1,""))</f>
+        <f>IF(B28="","",IF(MONTH(B28+1)=$C$2,B28+1,""))</f>
         <v/>
       </c>
       <c r="C29" s="9">
@@ -1406,25 +1461,25 @@
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="B30" s="8">
-        <f>IF(B29="","",IF(MONTH(B29+1)=$C$5,B29+1,""))</f>
+        <f>IF(B29="","",IF(MONTH(B29+1)=$C$2,B29+1,""))</f>
         <v/>
       </c>
       <c r="C30" s="9">
         <f>IF(B30="","",CHOOSE(WEEKDAY(B30,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
       <c r="F30" s="11">
         <f>IF(AND(D30&lt;&gt;"",E30&lt;&gt;""),E30-D30,"")</f>
         <v/>
       </c>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="13" t="n"/>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="16" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="B31" s="8">
-        <f>IF(B30="","",IF(MONTH(B30+1)=$C$5,B30+1,""))</f>
+        <f>IF(B30="","",IF(MONTH(B30+1)=$C$2,B30+1,""))</f>
         <v/>
       </c>
       <c r="C31" s="9">
@@ -1442,25 +1497,25 @@
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="B32" s="8">
-        <f>IF(B31="","",IF(MONTH(B31+1)=$C$5,B31+1,""))</f>
+        <f>IF(B31="","",IF(MONTH(B31+1)=$C$2,B31+1,""))</f>
         <v/>
       </c>
       <c r="C32" s="9">
         <f>IF(B32="","",CHOOSE(WEEKDAY(B32,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="10" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
       <c r="F32" s="11">
         <f>IF(AND(D32&lt;&gt;"",E32&lt;&gt;""),E32-D32,"")</f>
         <v/>
       </c>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="13" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="16" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="B33" s="8">
-        <f>IF(B32="","",IF(MONTH(B32+1)=$C$5,B32+1,""))</f>
+        <f>IF(B32="","",IF(MONTH(B32+1)=$C$2,B32+1,""))</f>
         <v/>
       </c>
       <c r="C33" s="9">
@@ -1478,25 +1533,25 @@
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="B34" s="8">
-        <f>IF(B33="","",IF(MONTH(B33+1)=$C$5,B33+1,""))</f>
+        <f>IF(B33="","",IF(MONTH(B33+1)=$C$2,B33+1,""))</f>
         <v/>
       </c>
       <c r="C34" s="9">
         <f>IF(B34="","",CHOOSE(WEEKDAY(B34,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
         <v/>
       </c>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
+      <c r="D34" s="14" t="n"/>
+      <c r="E34" s="14" t="n"/>
       <c r="F34" s="11">
         <f>IF(AND(D34&lt;&gt;"",E34&lt;&gt;""),E34-D34,"")</f>
         <v/>
       </c>
-      <c r="G34" s="12" t="n"/>
-      <c r="H34" s="13" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="16" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="B35" s="8">
-        <f>IF(B34="","",IF(MONTH(B34+1)=$C$5,B34+1,""))</f>
+        <f>IF(B34="","",IF(MONTH(B34+1)=$C$2,B34+1,""))</f>
         <v/>
       </c>
       <c r="C35" s="9">
@@ -1512,205 +1567,144 @@
       <c r="G35" s="12" t="n"/>
       <c r="H35" s="13" t="n"/>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="8">
-        <f>IF(B35="","",IF(MONTH(B35+1)=$C$5,B35+1,""))</f>
-        <v/>
-      </c>
-      <c r="C36" s="9">
-        <f>IF(B36="","",CHOOSE(WEEKDAY(B36,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
-        <v/>
-      </c>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="11">
-        <f>IF(AND(D36&lt;&gt;"",E36&lt;&gt;""),E36-D36,"")</f>
-        <v/>
-      </c>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="13" t="n"/>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="8">
-        <f>IF(B36="","",IF(MONTH(B36+1)=$C$5,B36+1,""))</f>
-        <v/>
-      </c>
-      <c r="C37" s="9">
-        <f>IF(B37="","",CHOOSE(WEEKDAY(B37,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
-        <v/>
-      </c>
-      <c r="D37" s="10" t="n"/>
-      <c r="E37" s="10" t="n"/>
-      <c r="F37" s="11">
-        <f>IF(AND(D37&lt;&gt;"",E37&lt;&gt;""),E37-D37,"")</f>
-        <v/>
-      </c>
-      <c r="G37" s="12" t="n"/>
-      <c r="H37" s="13" t="n"/>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="B38" s="8">
-        <f>IF(B37="","",IF(MONTH(B37+1)=$C$5,B37+1,""))</f>
-        <v/>
-      </c>
-      <c r="C38" s="9">
-        <f>IF(B38="","",CHOOSE(WEEKDAY(B38,1),"الأحد","الاثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت"))</f>
-        <v/>
-      </c>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="11">
-        <f>IF(AND(D38&lt;&gt;"",E38&lt;&gt;""),E38-D38,"")</f>
-        <v/>
-      </c>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="10" customHeight="1"/>
-    <row r="40" ht="32" customHeight="1">
-      <c r="B40" s="14" t="inlineStr">
+    <row r="36" ht="22" customHeight="1"/>
+    <row r="37">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>ملخص الشهر</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>أيام الشهر الكاملة</t>
-        </is>
-      </c>
-      <c r="F41" s="16">
-        <f>DAY(DATE($F$5,$C$5+1,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="B42" s="17" t="inlineStr">
+    <row r="38" ht="27" customHeight="1">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>أيام الحضور</t>
         </is>
       </c>
-      <c r="F42" s="18">
-        <f>COUNTIF(G8:G38,"حاضر")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="B43" s="19" t="inlineStr">
+      <c r="F38" s="19">
+        <f>COUNTIF(G5:G35,"حضور")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="27" customHeight="1">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>أيام الغياب</t>
         </is>
       </c>
-      <c r="F43" s="20">
-        <f>COUNTIF(G8:G38,"غائب")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="B44" s="21" t="inlineStr">
+      <c r="F39" s="21">
+        <f>COUNTIF(G5:G35,"غياب")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="27" customHeight="1">
+      <c r="B40" s="22" t="inlineStr">
         <is>
           <t>أيام الإجازة</t>
         </is>
       </c>
-      <c r="F44" s="22">
-        <f>COUNTIF(G8:G38,"إجازة")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="B45" s="23" t="inlineStr">
+      <c r="F40" s="23">
+        <f>COUNTIF(G5:G35,"إجازة")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="27" customHeight="1">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>أيام الترك</t>
         </is>
       </c>
-      <c r="F45" s="24">
-        <f>COUNTIF(G8:G38,"ترك")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="B46" s="25" t="inlineStr">
-        <is>
-          <t>الإجازات الرسمية</t>
-        </is>
-      </c>
-      <c r="F46" s="26">
-        <f>COUNTIF(G8:G38,"إجازة رسمية")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="28" customHeight="1">
-      <c r="B47" s="27" t="inlineStr">
+      <c r="F41" s="25">
+        <f>COUNTIF(G5:G35,"ترك")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="27" customHeight="1">
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>مستأذن</t>
+        </is>
+      </c>
+      <c r="F42" s="27">
+        <f>COUNTIF(G5:G35,"مستأذن")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="27" customHeight="1">
+      <c r="B43" s="28" t="inlineStr">
         <is>
           <t>إجمالي ساعات العمل</t>
         </is>
       </c>
-      <c r="F47" s="28">
-        <f>IFERROR(SUM(F8:F38),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="28" customHeight="1"/>
-    <row r="49" ht="28" customHeight="1">
-      <c r="B49" s="29" t="inlineStr">
-        <is>
-          <t>ملاحظة: عند تغيير الشهر تتحدث التواريخ تلقائياً — أدخل وقت الدخول والخروج بصيغة  HH:MM</t>
-        </is>
-      </c>
-    </row>
+      <c r="F43" s="29">
+        <f>IFERROR(SUM(F5:F35),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="27" customHeight="1"/>
+    <row r="45" ht="27" customHeight="1"/>
+    <row r="46" ht="27" customHeight="1"/>
+    <row r="47" ht="27" customHeight="1"/>
+    <row r="48" ht="27" customHeight="1"/>
+    <row r="49" ht="27" customHeight="1"/>
+    <row r="50" ht="27" customHeight="1"/>
+    <row r="51" ht="27" customHeight="1"/>
+    <row r="52" ht="27" customHeight="1"/>
+    <row r="53" ht="27" customHeight="1"/>
+    <row r="54" ht="27" customHeight="1"/>
+    <row r="55" ht="27" customHeight="1"/>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="B40:H40"/>
+  <mergeCells count="17">
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:E41"/>
     <mergeCell ref="F42:H42"/>
-    <mergeCell ref="F45:H45"/>
-    <mergeCell ref="B49:H49"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="F39:H39"/>
+    <mergeCell ref="B43:E43"/>
     <mergeCell ref="F41:H41"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F40:H40"/>
     <mergeCell ref="F43:H43"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="F44:H44"/>
     <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="G3:H3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:H38">
+  <conditionalFormatting sqref="B5:H35">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>=$G8="حاضر"</formula>
+      <formula>=$G5="حضور"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>=$G8="غائب"</formula>
+      <formula>=$G5="غياب"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>=$G8="إجازة"</formula>
+      <formula>=$G5="ترك"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>=$G8="ترك"</formula>
+      <formula>=$G5="إجازة"</formula>
     </cfRule>
     <cfRule type="expression" priority="5" dxfId="4">
-      <formula>=$G8="إجازة رسمية"</formula>
+      <formula>=$G5="مستأذن"</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="5">
-      <formula>=AND($B8&lt;&gt;"",OR(WEEKDAY($B8,1)=6,WEEKDAY($B8,1)=7))</formula>
+      <formula>=$G5="عطلة رسمية"</formula>
     </cfRule>
     <cfRule type="expression" priority="7" dxfId="6">
-      <formula>=$B8=""</formula>
+      <formula>=OR(WEEKDAY($B5,1)=6,WEEKDAY($B5,1)=7)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="7">
+      <formula>=$B5=""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="اختر الشهر" prompt="أدخل رقم الشهر (1 إلى 12)" type="list">
+    <dataValidation sqref="C2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
     </dataValidation>
-    <dataValidation sqref="G8:G38" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="خطأ في الإدخال" error="الرجاء الاختيار من القائمة المنسدلة" promptTitle="الحالة" prompt="اختر: حاضر | غائب | إجازة | ترك | إجازة رسمية" type="list">
-      <formula1>"حاضر,غائب,إجازة,ترك,إجازة رسمية"</formula1>
+    <dataValidation sqref="G5:G35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="الحالة" prompt="حضور | غياب | ترك | إجازة | مستأذن | عطلة رسمية" type="list">
+      <formula1>"حضور,غياب,ترك,إجازة,مستأذن,عطلة رسمية"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>